<commit_message>
dicionário + módulo A
</commit_message>
<xml_diff>
--- a/documentos/modelo_dicionario_de_dados.xlsx
+++ b/documentos/modelo_dicionario_de_dados.xlsx
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="326" uniqueCount="121">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="570" uniqueCount="170">
   <si>
     <t xml:space="preserve">MODELO DE DICIONÁRIO DE DADOS</t>
   </si>
@@ -190,6 +190,153 @@
   </si>
   <si>
     <t xml:space="preserve">modelo  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chave primaria de identificação da categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome da categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funcionario.id</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funcionário responsável pelo cadastro da categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funcionario.id_cargo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cargo do funcionário responsável</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cadastro do status da categoria (0,1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATETIME ('now','localtime')</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data de cadastro da categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">servico</t>
+  </si>
+  <si>
+    <t xml:space="preserve">id_servicos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chave primaria de identificação do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_servicos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoria.id_categoria</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoria relacionada ao serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preco</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preço do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">horas_trabalho</t>
+  </si>
+  <si>
+    <t xml:space="preserve">REAL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quantidade de horas estimadas para execução do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funcionário responsável pelo cadastro do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cadastro do status do serviço (0,1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data de cadastro do serviço</t>
+  </si>
+  <si>
+    <t xml:space="preserve">peca</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chave primaria de identificação da peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome da peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">categoria relacionada à peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preco_compra</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preço de compra da peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preco_venda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preço de venda da peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">estoque_atual</t>
+  </si>
+  <si>
+    <t xml:space="preserve">quantidade atual disponível em estoque</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funcionário responsável pelo cadastro da peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cadastro do status da peça (0,1)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data de cadastro da peça</t>
+  </si>
+  <si>
+    <t xml:space="preserve">forma_pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">chave primaria de identificação da forma de pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome_forma_pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">nome da forma de pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">funcionário responsável pelo cadastro da forma de pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">data de cadastro da forma de pagamento</t>
+  </si>
+  <si>
+    <t xml:space="preserve">cadastro do status da forma de pagamento (0,1)</t>
   </si>
   <si>
     <t xml:space="preserve">INSTRUÇÕES E EXEMPLO PRÁTICO</t>
@@ -538,12 +685,8 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="23">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -551,28 +694,28 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -583,14 +726,6 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -599,12 +734,20 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -617,6 +760,22 @@
     </xf>
     <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -871,17 +1030,17 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H59"/>
+  <dimension ref="A1:H78"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="2" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="2" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="4" style="1" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="30"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="45"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="0" width="11.53"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="16384" min="16384" style="2" width="11.53"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -955,102 +1114,96 @@
       <c r="B10" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C10" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="10" t="s">
+      <c r="C10" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E10" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F10" s="9" t="s">
+      <c r="E10" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F10" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G10" s="8"/>
-      <c r="H10" s="11" t="s">
+      <c r="H10" s="9" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="12" t="s">
+      <c r="A11" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B11" s="12" t="s">
+      <c r="B11" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="C11" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="14"/>
-      <c r="E11" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F11" s="13"/>
-      <c r="G11" s="12"/>
-      <c r="H11" s="15"/>
+      <c r="D11" s="11"/>
+      <c r="E11" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F11" s="10"/>
+      <c r="G11" s="10"/>
+      <c r="H11" s="11"/>
     </row>
     <row r="12" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B12" s="0" t="s">
+      <c r="B12" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C12" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="16" t="s">
+      <c r="C12" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E12" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F12" s="13" t="s">
+      <c r="E12" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="G12" s="0"/>
-      <c r="H12" s="0"/>
     </row>
     <row r="13" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B13" s="0" t="s">
+      <c r="B13" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C13" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F13" s="16" t="n">
+      <c r="C13" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F13" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G13" s="0"/>
-      <c r="H13" s="0"/>
     </row>
     <row r="14" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B14" s="0" t="s">
+      <c r="B14" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F14" s="16" t="s">
+      <c r="D14" s="12"/>
+      <c r="E14" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F14" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="G14" s="0"/>
-      <c r="H14" s="0"/>
     </row>
     <row r="15" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="8" t="s">
@@ -1059,140 +1212,131 @@
       <c r="B15" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="10" t="s">
+      <c r="C15" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E15" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F15" s="9" t="s">
+      <c r="E15" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F15" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G15" s="8"/>
-      <c r="H15" s="11" t="s">
+      <c r="H15" s="9" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
+      <c r="A16" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="B16" s="12" t="s">
+      <c r="B16" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="C16" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F16" s="13"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="15"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F16" s="10"/>
+      <c r="G16" s="10"/>
+      <c r="H16" s="11"/>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C17" s="16" t="s">
+      <c r="C17" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F17" s="13" t="s">
+      <c r="D17" s="12"/>
+      <c r="E17" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F17" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="G17" s="0"/>
-      <c r="H17" s="0"/>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="0" t="s">
+      <c r="B18" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C18" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F18" s="16" t="n">
+      <c r="C18" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F18" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="G18" s="0"/>
-      <c r="H18" s="0" t="s">
+      <c r="H18" s="1" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B19" s="0" t="s">
+      <c r="B19" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="C19" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D19" s="16" t="s">
+      <c r="C19" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D19" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E19" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F19" s="16"/>
-      <c r="G19" s="0"/>
-      <c r="H19" s="0"/>
+      <c r="E19" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F19" s="12"/>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="0" t="s">
+      <c r="B20" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="C20" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D20" s="16" t="s">
+      <c r="C20" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D20" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E20" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F20" s="16"/>
-      <c r="G20" s="0"/>
-      <c r="H20" s="0"/>
+      <c r="E20" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F20" s="12"/>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B21" s="0" t="s">
+      <c r="B21" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C21" s="16" t="s">
+      <c r="C21" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F21" s="16"/>
-      <c r="G21" s="0"/>
-      <c r="H21" s="0"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F21" s="12"/>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="8" t="s">
@@ -1201,190 +1345,174 @@
       <c r="B22" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C22" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D22" s="10" t="s">
+      <c r="C22" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E22" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F22" s="9" t="s">
+      <c r="E22" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F22" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G22" s="8"/>
-      <c r="H22" s="11" t="s">
+      <c r="H22" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
+      <c r="A23" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="12" t="s">
+      <c r="B23" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="13" t="s">
+      <c r="C23" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D23" s="14"/>
-      <c r="E23" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F23" s="13"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="15"/>
+      <c r="D23" s="11"/>
+      <c r="E23" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F23" s="10"/>
+      <c r="G23" s="10"/>
+      <c r="H23" s="11"/>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="8" t="s">
         <v>38</v>
       </c>
-      <c r="B24" s="0" t="s">
+      <c r="B24" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="C24" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D24" s="16" t="s">
+      <c r="C24" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D24" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E24" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F24" s="16"/>
-      <c r="G24" s="0"/>
-      <c r="H24" s="0"/>
+      <c r="E24" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F24" s="12"/>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12" t="s">
+      <c r="A25" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="0" t="s">
+      <c r="B25" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="C25" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D25" s="16" t="s">
+      <c r="C25" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E25" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F25" s="16"/>
-      <c r="G25" s="0"/>
-      <c r="H25" s="0"/>
+      <c r="E25" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F25" s="12"/>
     </row>
     <row r="26" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12" t="s">
+      <c r="A26" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B26" s="0" t="s">
+      <c r="B26" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="C26" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D26" s="16" t="s">
+      <c r="C26" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D26" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="E26" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F26" s="16"/>
-      <c r="G26" s="0"/>
-      <c r="H26" s="0"/>
+      <c r="E26" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F26" s="12"/>
     </row>
     <row r="27" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
+      <c r="A27" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B27" s="0" t="s">
+      <c r="B27" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="C27" s="13" t="s">
+      <c r="C27" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D27" s="16"/>
-      <c r="E27" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F27" s="16"/>
-      <c r="G27" s="0"/>
-      <c r="H27" s="0"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F27" s="12"/>
     </row>
     <row r="28" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="12" t="s">
+      <c r="A28" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B28" s="0" t="s">
+      <c r="B28" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="C28" s="16" t="s">
+      <c r="C28" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16" t="s">
+      <c r="D28" s="12"/>
+      <c r="E28" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="F28" s="16"/>
-      <c r="G28" s="0"/>
-      <c r="H28" s="0"/>
+      <c r="F28" s="12"/>
     </row>
     <row r="29" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="12" t="s">
+      <c r="A29" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B29" s="0" t="s">
+      <c r="B29" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="C29" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F29" s="16"/>
-      <c r="G29" s="0"/>
-      <c r="H29" s="0"/>
+      <c r="C29" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F29" s="12"/>
     </row>
     <row r="30" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="12" t="s">
+      <c r="A30" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B30" s="0" t="s">
+      <c r="B30" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C30" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F30" s="16"/>
-      <c r="G30" s="0"/>
-      <c r="H30" s="0"/>
+      <c r="C30" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F30" s="12"/>
     </row>
     <row r="31" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="12" t="s">
+      <c r="A31" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B31" s="0" t="s">
+      <c r="B31" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C31" s="13" t="s">
+      <c r="C31" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D31" s="16"/>
-      <c r="E31" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F31" s="16"/>
-      <c r="G31" s="0"/>
-      <c r="H31" s="0"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F31" s="12"/>
     </row>
     <row r="32" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="8" t="s">
@@ -1393,60 +1521,60 @@
       <c r="B32" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C32" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D32" s="10" t="s">
+      <c r="C32" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D32" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E32" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F32" s="9" t="s">
+      <c r="E32" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F32" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G32" s="8"/>
-      <c r="H32" s="11" t="s">
+      <c r="H32" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="12" t="s">
+      <c r="A33" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="B33" s="12" t="s">
+      <c r="B33" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="C33" s="13" t="s">
+      <c r="C33" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D33" s="14"/>
-      <c r="E33" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F33" s="13" t="s">
+      <c r="D33" s="11"/>
+      <c r="E33" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F33" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="G33" s="12"/>
-      <c r="H33" s="15"/>
+      <c r="G33" s="10"/>
+      <c r="H33" s="11"/>
     </row>
     <row r="34" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="12" t="s">
+      <c r="A34" s="10" t="s">
         <v>48</v>
       </c>
       <c r="B34" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C34" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D34" s="10"/>
-      <c r="E34" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F34" s="9"/>
+      <c r="C34" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" s="9"/>
+      <c r="E34" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F34" s="8"/>
       <c r="G34" s="8"/>
-      <c r="H34" s="11"/>
+      <c r="H34" s="9"/>
     </row>
     <row r="35" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="8" t="s">
@@ -1455,390 +1583,1064 @@
       <c r="B35" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="C35" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D35" s="10" t="s">
+      <c r="C35" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D35" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="E35" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="F35" s="9" t="s">
+      <c r="E35" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="F35" s="8" t="s">
         <v>21</v>
       </c>
       <c r="G35" s="8"/>
-      <c r="H35" s="11" t="s">
+      <c r="H35" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A36" s="12" t="s">
+      <c r="A36" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B36" s="12" t="s">
+      <c r="B36" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="C36" s="13" t="s">
+      <c r="C36" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="F36" s="13"/>
-      <c r="G36" s="12"/>
-      <c r="H36" s="15"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="F36" s="10"/>
+      <c r="G36" s="10"/>
+      <c r="H36" s="11"/>
     </row>
     <row r="37" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A37" s="12" t="s">
+      <c r="A37" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="B37" s="0" t="s">
+      <c r="B37" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C37" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D37" s="16"/>
-      <c r="E37" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F37" s="16"/>
-      <c r="G37" s="0"/>
-      <c r="H37" s="0"/>
+      <c r="C37" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F37" s="12"/>
     </row>
     <row r="38" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
+      <c r="A38" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B38" s="0" t="s">
+      <c r="B38" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C38" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D38" s="16" t="s">
+      <c r="C38" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D38" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E38" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F38" s="16" t="s">
+      <c r="E38" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F38" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="G38" s="0"/>
-      <c r="H38" s="11" t="s">
+      <c r="H38" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
+      <c r="A39" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B39" s="0" t="s">
+      <c r="B39" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C39" s="16" t="s">
+      <c r="C39" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D39" s="16"/>
-      <c r="E39" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F39" s="16"/>
-      <c r="G39" s="0"/>
-      <c r="H39" s="0"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F39" s="12"/>
     </row>
     <row r="40" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+      <c r="A40" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B40" s="0" t="s">
+      <c r="B40" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C40" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D40" s="16"/>
-      <c r="E40" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F40" s="16"/>
-      <c r="G40" s="0"/>
-      <c r="H40" s="0"/>
+      <c r="C40" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D40" s="12"/>
+      <c r="E40" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F40" s="12"/>
     </row>
     <row r="41" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
+      <c r="A41" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B41" s="12" t="s">
+      <c r="B41" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C41" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D41" s="14" t="s">
+      <c r="C41" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D41" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="E41" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F41" s="13"/>
-      <c r="G41" s="12"/>
-      <c r="H41" s="15"/>
+      <c r="E41" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F41" s="10"/>
+      <c r="G41" s="10"/>
+      <c r="H41" s="11"/>
     </row>
     <row r="42" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
+      <c r="A42" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B42" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="C42" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D42" s="10" t="s">
+      <c r="C42" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D42" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E42" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F42" s="9"/>
+      <c r="E42" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F42" s="8"/>
       <c r="G42" s="8"/>
-      <c r="H42" s="11"/>
+      <c r="H42" s="9"/>
     </row>
     <row r="43" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
+      <c r="A43" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B43" s="0" t="s">
+      <c r="B43" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="C43" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D43" s="16" t="s">
+      <c r="C43" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D43" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="E43" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F43" s="16" t="s">
+      <c r="E43" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F43" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="G43" s="0"/>
-      <c r="H43" s="11" t="s">
+      <c r="H43" s="9" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
+      <c r="A44" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B44" s="0" t="s">
+      <c r="B44" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="C44" s="16" t="s">
+      <c r="C44" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D44" s="16"/>
-      <c r="E44" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F44" s="16"/>
-      <c r="G44" s="0"/>
-      <c r="H44" s="0"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F44" s="12"/>
     </row>
     <row r="45" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
+      <c r="A45" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B45" s="0" t="s">
+      <c r="B45" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C45" s="16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D45" s="16"/>
-      <c r="E45" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F45" s="16"/>
-      <c r="G45" s="0"/>
-      <c r="H45" s="0"/>
+      <c r="C45" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D45" s="12"/>
+      <c r="E45" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F45" s="12"/>
     </row>
     <row r="46" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
+      <c r="A46" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B46" s="12" t="s">
+      <c r="B46" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="C46" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D46" s="14" t="s">
+      <c r="C46" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D46" s="11" t="s">
         <v>26</v>
       </c>
-      <c r="E46" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F46" s="13"/>
-      <c r="G46" s="12"/>
-      <c r="H46" s="15"/>
+      <c r="E46" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F46" s="10"/>
+      <c r="G46" s="10"/>
+      <c r="H46" s="11"/>
     </row>
     <row r="47" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
+      <c r="A47" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B47" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="C47" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D47" s="10" t="s">
+      <c r="C47" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D47" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="E47" s="16" t="s">
-        <v>20</v>
-      </c>
-      <c r="F47" s="9"/>
+      <c r="E47" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F47" s="8"/>
       <c r="G47" s="8"/>
-      <c r="H47" s="11"/>
+      <c r="H47" s="9"/>
     </row>
     <row r="48" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A48" s="8"/>
-      <c r="B48" s="8"/>
-      <c r="C48" s="9"/>
-      <c r="D48" s="10"/>
-      <c r="E48" s="10"/>
-      <c r="F48" s="9"/>
-      <c r="G48" s="8"/>
-      <c r="H48" s="11"/>
+      <c r="A48" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B48" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C48" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D48" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E48" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F48" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G48" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H48" s="13" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="49" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A49" s="12"/>
-      <c r="B49" s="12"/>
-      <c r="C49" s="13"/>
-      <c r="D49" s="14"/>
-      <c r="E49" s="14"/>
-      <c r="F49" s="13"/>
-      <c r="G49" s="12"/>
-      <c r="H49" s="15"/>
+      <c r="A49" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B49" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="C49" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D49" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E49" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F49" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G49" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H49" s="13" t="s">
+        <v>61</v>
+      </c>
     </row>
     <row r="50" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A50" s="8"/>
-      <c r="B50" s="8"/>
-      <c r="C50" s="9"/>
-      <c r="D50" s="10"/>
-      <c r="E50" s="10"/>
-      <c r="F50" s="9"/>
-      <c r="G50" s="8"/>
-      <c r="H50" s="11"/>
+      <c r="A50" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B50" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C50" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D50" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E50" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F50" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G50" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="H50" s="13" t="s">
+        <v>63</v>
+      </c>
     </row>
     <row r="51" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A51" s="12"/>
-      <c r="B51" s="12"/>
-      <c r="C51" s="13"/>
-      <c r="D51" s="14"/>
-      <c r="E51" s="14"/>
-      <c r="F51" s="13"/>
-      <c r="G51" s="12"/>
-      <c r="H51" s="15"/>
+      <c r="A51" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B51" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C51" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D51" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E51" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F51" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G51" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="H51" s="13" t="s">
+        <v>65</v>
+      </c>
     </row>
     <row r="52" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A52" s="8"/>
-      <c r="B52" s="8"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="10"/>
-      <c r="E52" s="10"/>
-      <c r="F52" s="9"/>
-      <c r="G52" s="8"/>
-      <c r="H52" s="11"/>
+      <c r="A52" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B52" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C52" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D52" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E52" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F52" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G52" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H52" s="13" t="s">
+        <v>66</v>
+      </c>
     </row>
     <row r="53" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A53" s="12"/>
-      <c r="B53" s="12"/>
-      <c r="C53" s="13"/>
-      <c r="D53" s="14"/>
-      <c r="E53" s="14"/>
-      <c r="F53" s="13"/>
-      <c r="G53" s="12"/>
-      <c r="H53" s="15"/>
+      <c r="A53" s="13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B53" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C53" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D53" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E53" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F53" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G53" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H53" s="13" t="s">
+        <v>68</v>
+      </c>
     </row>
     <row r="54" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A54" s="8"/>
-      <c r="B54" s="8"/>
-      <c r="C54" s="9"/>
-      <c r="D54" s="10"/>
-      <c r="E54" s="10"/>
-      <c r="F54" s="9"/>
-      <c r="G54" s="8"/>
-      <c r="H54" s="11"/>
+      <c r="A54" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B54" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="C54" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D54" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E54" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F54" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G54" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H54" s="13" t="s">
+        <v>71</v>
+      </c>
     </row>
     <row r="55" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A55" s="12"/>
-      <c r="B55" s="12"/>
-      <c r="C55" s="13"/>
-      <c r="D55" s="14"/>
-      <c r="E55" s="14"/>
-      <c r="F55" s="13"/>
-      <c r="G55" s="12"/>
-      <c r="H55" s="15"/>
+      <c r="A55" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B55" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="C55" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D55" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E55" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F55" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G55" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H55" s="13" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="56" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A56" s="8"/>
-      <c r="B56" s="8"/>
-      <c r="C56" s="9"/>
-      <c r="D56" s="10"/>
-      <c r="E56" s="10"/>
-      <c r="F56" s="9"/>
-      <c r="G56" s="8"/>
-      <c r="H56" s="11"/>
+      <c r="A56" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B56" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C56" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D56" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F56" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G56" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="H56" s="13" t="s">
+        <v>75</v>
+      </c>
     </row>
     <row r="57" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A57" s="12"/>
-      <c r="B57" s="12"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="14"/>
-      <c r="E57" s="14"/>
-      <c r="F57" s="13"/>
-      <c r="G57" s="12"/>
-      <c r="H57" s="15"/>
+      <c r="A57" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B57" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="C57" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D57" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E57" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F57" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G57" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H57" s="13" t="s">
+        <v>77</v>
+      </c>
     </row>
     <row r="58" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A58" s="8"/>
-      <c r="B58" s="8"/>
-      <c r="C58" s="9"/>
-      <c r="D58" s="10"/>
-      <c r="E58" s="10"/>
-      <c r="F58" s="9"/>
-      <c r="G58" s="8"/>
-      <c r="H58" s="11"/>
+      <c r="A58" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B58" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="C58" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="D58" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E58" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F58" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G58" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H58" s="13" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="59" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A59" s="12"/>
-      <c r="B59" s="12"/>
-      <c r="C59" s="13"/>
-      <c r="D59" s="14"/>
-      <c r="E59" s="14"/>
-      <c r="F59" s="13"/>
-      <c r="G59" s="12"/>
-      <c r="H59" s="15"/>
+      <c r="A59" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B59" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C59" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D59" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E59" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F59" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G59" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="H59" s="13" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B60" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C60" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D60" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E60" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F60" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G60" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="H60" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B61" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C61" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D61" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E61" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F61" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G61" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H61" s="13" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="B62" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C62" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D62" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E62" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F62" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G62" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H62" s="13" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B63" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C63" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D63" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E63" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F63" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G63" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H63" s="13" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B64" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="C64" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D64" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E64" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F64" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G64" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H64" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B65" s="13" t="s">
+        <v>57</v>
+      </c>
+      <c r="C65" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D65" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E65" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F65" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G65" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="H65" s="13" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B66" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="C66" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D66" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E66" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F66" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G66" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H66" s="13" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B67" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="C67" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D67" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E67" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F67" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G67" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H67" s="13" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B68" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="C68" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D68" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E68" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F68" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G68" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H68" s="13" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B69" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C69" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D69" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E69" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F69" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G69" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="H69" s="13" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B70" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C70" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D70" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E70" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F70" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G70" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="H70" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B71" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C71" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D71" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E71" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F71" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G71" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H71" s="13" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="B72" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C72" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D72" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E72" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F72" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G72" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H72" s="13" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B73" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="C73" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D73" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="E73" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F73" s="13" t="s">
+        <v>21</v>
+      </c>
+      <c r="G73" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H73" s="13" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A74" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B74" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C74" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D74" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E74" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F74" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G74" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H74" s="13" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B75" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="C75" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D75" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E75" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F75" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G75" s="13" t="s">
+        <v>62</v>
+      </c>
+      <c r="H75" s="13" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A76" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B76" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C76" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D76" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="E76" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F76" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="G76" s="13" t="s">
+        <v>64</v>
+      </c>
+      <c r="H76" s="13" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A77" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B77" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C77" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D77" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E77" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F77" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G77" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H77" s="13" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A78" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="B78" s="13" t="s">
+        <v>28</v>
+      </c>
+      <c r="C78" s="13" t="s">
+        <v>18</v>
+      </c>
+      <c r="D78" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="E78" s="13" t="s">
+        <v>20</v>
+      </c>
+      <c r="F78" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="G78" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="H78" s="13" t="s">
+        <v>104</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C11 C15:C16 C22:C23 C27 C31:C36 C41:C42 C46:C59" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="C10:C11 C15:C16 C22:C23 C27 C31:C36 C41:C42 C46:C47" type="list">
       <formula1>Validações!$A$1:$A$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D10:D11 D15:D16 D22:D23 D32:D36 D41:D42 D46:D59" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="D10:D11 D15:D16 D22:D23 D32:D36 D41:D42 D46:D47" type="list">
       <formula1>Validações!$B$1:$B$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E11 E15:E16 E22:E23 E32:E33 E35:E36 E48:E59" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="E10:E11 E15:E16 E22:E23 E32:E33 E35:E36" type="list">
       <formula1>Validações!$C$1:$C$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -1861,101 +2663,101 @@
   <dimension ref="A1:I25"/>
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="22"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="17"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="30"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="45"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="27"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="22"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="2" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="2" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="2" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="2" width="45"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="19.7" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="3" t="s">
-        <v>56</v>
+      <c r="A1" s="14" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="4" t="s">
-        <v>57</v>
+      <c r="A2" s="15" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="B4" s="18" t="s">
-        <v>59</v>
+      <c r="A4" s="16" t="s">
+        <v>107</v>
+      </c>
+      <c r="B4" s="17" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="B5" s="18" t="s">
-        <v>61</v>
+      <c r="A5" s="16" t="s">
+        <v>109</v>
+      </c>
+      <c r="B5" s="17" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="17" t="s">
-        <v>62</v>
-      </c>
-      <c r="B6" s="18" t="s">
-        <v>63</v>
+      <c r="A6" s="16" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" s="17" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="17" t="s">
-        <v>64</v>
-      </c>
-      <c r="B7" s="18" t="s">
-        <v>65</v>
+      <c r="A7" s="16" t="s">
+        <v>113</v>
+      </c>
+      <c r="B7" s="17" t="s">
+        <v>114</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>67</v>
+      <c r="A8" s="16" t="s">
+        <v>115</v>
+      </c>
+      <c r="B8" s="17" t="s">
+        <v>116</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="17" t="s">
-        <v>68</v>
-      </c>
-      <c r="B9" s="18" t="s">
-        <v>69</v>
+      <c r="A9" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>118</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="17" t="s">
-        <v>70</v>
-      </c>
-      <c r="B10" s="18" t="s">
-        <v>71</v>
+      <c r="A10" s="16" t="s">
+        <v>119</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>120</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="17" t="s">
-        <v>72</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>73</v>
+      <c r="A11" s="16" t="s">
+        <v>121</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="17" t="s">
-        <v>74</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>75</v>
+      <c r="A12" s="16" t="s">
+        <v>123</v>
+      </c>
+      <c r="B12" s="17" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="19" t="s">
-        <v>76</v>
+      <c r="A14" s="18" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="24.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1963,13 +2765,13 @@
         <v>8</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>77</v>
+        <v>126</v>
       </c>
       <c r="C16" s="7" t="s">
         <v>10</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>78</v>
+        <v>127</v>
       </c>
       <c r="E16" s="7" t="s">
         <v>11</v>
@@ -1978,256 +2780,256 @@
         <v>12</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>79</v>
+        <v>128</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>80</v>
+        <v>129</v>
       </c>
       <c r="I16" s="7" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="E17" s="14" t="s">
+      <c r="A17" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="B17" s="19" t="s">
+        <v>131</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E17" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F17" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="G17" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="H17" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="I17" s="15" t="s">
-        <v>86</v>
+      <c r="F17" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="G17" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="H17" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="I17" s="20" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="B18" s="8" t="s">
-        <v>87</v>
-      </c>
-      <c r="C18" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="E18" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="F18" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G18" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="H18" s="8" t="s">
-        <v>91</v>
+      <c r="A18" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="B18" s="21" t="s">
+        <v>136</v>
+      </c>
+      <c r="C18" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D18" s="9" t="s">
+        <v>138</v>
+      </c>
+      <c r="E18" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="F18" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G18" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="H18" s="21" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="D19" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="E19" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="F19" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="G19" s="13" t="s">
-        <v>85</v>
-      </c>
-      <c r="H19" s="12" t="s">
-        <v>93</v>
+      <c r="A19" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="B19" s="19" t="s">
+        <v>141</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E19" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="F19" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>134</v>
+      </c>
+      <c r="H19" s="19" t="s">
+        <v>142</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="B20" s="8" t="s">
-        <v>94</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>95</v>
-      </c>
-      <c r="D20" s="10" t="s">
-        <v>85</v>
-      </c>
-      <c r="E20" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G20" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="H20" s="8" t="s">
-        <v>96</v>
+      <c r="A20" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="B20" s="21" t="s">
+        <v>143</v>
+      </c>
+      <c r="C20" s="8" t="s">
+        <v>144</v>
+      </c>
+      <c r="D20" s="9" t="s">
+        <v>134</v>
+      </c>
+      <c r="E20" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="F20" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G20" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="H20" s="21" t="s">
+        <v>145</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="C21" s="13" t="s">
-        <v>88</v>
-      </c>
-      <c r="D21" s="14" t="s">
-        <v>89</v>
-      </c>
-      <c r="E21" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="F21" s="14" t="s">
+      <c r="A21" s="19" t="s">
+        <v>130</v>
+      </c>
+      <c r="B21" s="19" t="s">
+        <v>146</v>
+      </c>
+      <c r="C21" s="10" t="s">
+        <v>137</v>
+      </c>
+      <c r="D21" s="11" t="s">
+        <v>138</v>
+      </c>
+      <c r="E21" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="F21" s="11" t="s">
         <v>46</v>
       </c>
-      <c r="G21" s="13" t="s">
-        <v>98</v>
-      </c>
-      <c r="H21" s="12" t="s">
-        <v>99</v>
+      <c r="G21" s="10" t="s">
+        <v>147</v>
+      </c>
+      <c r="H21" s="19" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8" t="s">
-        <v>81</v>
-      </c>
-      <c r="B22" s="8" t="s">
-        <v>100</v>
-      </c>
-      <c r="C22" s="9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>83</v>
-      </c>
-      <c r="E22" s="10" t="s">
+      <c r="A22" s="21" t="s">
+        <v>130</v>
+      </c>
+      <c r="B22" s="21" t="s">
+        <v>149</v>
+      </c>
+      <c r="C22" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="9" t="s">
+        <v>132</v>
+      </c>
+      <c r="E22" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="F22" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G22" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="H22" s="8" t="s">
-        <v>101</v>
-      </c>
-      <c r="I22" s="11" t="s">
-        <v>102</v>
+      <c r="F22" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G22" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="H22" s="21" t="s">
+        <v>150</v>
+      </c>
+      <c r="I22" s="22" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="C23" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D23" s="14" t="s">
-        <v>83</v>
-      </c>
-      <c r="E23" s="14" t="s">
+      <c r="A23" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="B23" s="19" t="s">
+        <v>149</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D23" s="11" t="s">
+        <v>132</v>
+      </c>
+      <c r="E23" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="F23" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="G23" s="13" t="s">
-        <v>84</v>
-      </c>
-      <c r="H23" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="I23" s="15" t="s">
-        <v>104</v>
+      <c r="F23" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="G23" s="10" t="s">
+        <v>133</v>
+      </c>
+      <c r="H23" s="19" t="s">
+        <v>134</v>
+      </c>
+      <c r="I23" s="20" t="s">
+        <v>153</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="B24" s="8" t="s">
-        <v>105</v>
-      </c>
-      <c r="C24" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="D24" s="10" t="s">
-        <v>106</v>
-      </c>
-      <c r="E24" s="10" t="s">
-        <v>90</v>
-      </c>
-      <c r="F24" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G24" s="9" t="s">
-        <v>85</v>
-      </c>
-      <c r="H24" s="8" t="s">
-        <v>107</v>
+      <c r="A24" s="21" t="s">
+        <v>152</v>
+      </c>
+      <c r="B24" s="21" t="s">
+        <v>154</v>
+      </c>
+      <c r="C24" s="8" t="s">
+        <v>137</v>
+      </c>
+      <c r="D24" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="E24" s="9" t="s">
+        <v>139</v>
+      </c>
+      <c r="F24" s="9" t="s">
+        <v>20</v>
+      </c>
+      <c r="G24" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="H24" s="21" t="s">
+        <v>156</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="C25" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D25" s="14" t="s">
-        <v>109</v>
-      </c>
-      <c r="E25" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="F25" s="14" t="s">
-        <v>20</v>
-      </c>
-      <c r="G25" s="13" t="s">
-        <v>110</v>
-      </c>
-      <c r="H25" s="12" t="s">
-        <v>111</v>
+      <c r="A25" s="19" t="s">
+        <v>152</v>
+      </c>
+      <c r="B25" s="19" t="s">
+        <v>157</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="D25" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="E25" s="11" t="s">
+        <v>139</v>
+      </c>
+      <c r="F25" s="11" t="s">
+        <v>20</v>
+      </c>
+      <c r="G25" s="10" t="s">
+        <v>159</v>
+      </c>
+      <c r="H25" s="19" t="s">
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -2250,76 +3052,76 @@
   <sheetFormatPr defaultColWidth="8.34375" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="B1" s="1" t="s">
+      <c r="A1" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="B2" s="1" t="s">
+      <c r="A2" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B2" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>114</v>
+      <c r="A3" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>163</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
-        <v>115</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>90</v>
+      <c r="A4" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>139</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
-        <v>116</v>
+      <c r="A5" s="2" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
-        <v>117</v>
+      <c r="A7" s="2" t="s">
+        <v>166</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
-        <v>95</v>
+      <c r="A8" s="2" t="s">
+        <v>144</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
-        <v>118</v>
+      <c r="A9" s="2" t="s">
+        <v>167</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
-        <v>119</v>
+      <c r="A10" s="2" t="s">
+        <v>168</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
-        <v>120</v>
+      <c r="A11" s="2" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>

</xml_diff>